<commit_message>
Added final modelling and handover notes
</commit_message>
<xml_diff>
--- a/checklists/Group_D_Week_3_Checklist_Updated.xlsx
+++ b/checklists/Group_D_Week_3_Checklist_Updated.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tpgtelecom-my.sharepoint.com/personal/bel_zhou_tpgtelecom_com_au/Documents/Documents/UNSW/Week 3/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/25a0eabcb09bfda7/Documents/Masters/2026-H5 - Data Science Project/ZZSC9020-Data-Science-Project-Group-D/checklists/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{08AB446C-B9BC-44E0-B8E5-D6C5B8EEF3B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="8_{08AB446C-B9BC-44E0-B8E5-D6C5B8EEF3B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{631D7C3F-4FEF-4696-901B-E30F13A9790A}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="960" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="13590" yWindow="1020" windowWidth="27645" windowHeight="19485" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Week 3 Checklist" sheetId="1" r:id="rId1"/>
@@ -345,53 +345,62 @@
       <sz val="22"/>
       <color rgb="FF17365D"/>
       <name val="Aptos Display"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="12"/>
       <color rgb="FF00A6A6"/>
       <name val="Aptos"/>
+      <family val="2"/>
     </font>
     <font>
       <i/>
       <sz val="10"/>
       <color rgb="FF64748B"/>
       <name val="Aptos"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Aptos"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF1F2937"/>
       <name val="Aptos"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="12"/>
       <color rgb="FFFFFFFF"/>
       <name val="Aptos"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FF17365D"/>
       <name val="Aptos"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="20"/>
       <color rgb="FF17365D"/>
       <name val="Aptos Display"/>
+      <family val="2"/>
     </font>
     <font>
       <i/>
       <sz val="11"/>
       <color rgb="FF64748B"/>
       <name val="Aptos"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="6">
@@ -833,7 +842,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:E36"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="29" customWidth="1"/>
@@ -842,7 +851,7 @@
     <col min="5" max="5" width="48" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="34" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
@@ -851,7 +860,7 @@
       <c r="D1" s="10"/>
       <c r="E1" s="10"/>
     </row>
-    <row r="2" spans="1:5" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
         <v>1</v>
       </c>
@@ -860,7 +869,7 @@
       <c r="D2" s="10"/>
       <c r="E2" s="10"/>
     </row>
-    <row r="3" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
         <v>2</v>
       </c>
@@ -869,14 +878,14 @@
       <c r="D3" s="10"/>
       <c r="E3" s="10"/>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="3"/>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
     </row>
-    <row r="5" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>3</v>
       </c>
@@ -893,7 +902,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="43" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" ht="42.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>8</v>
       </c>
@@ -910,7 +919,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="43" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" ht="42.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>8</v>
       </c>
@@ -927,7 +936,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="43" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" ht="42.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>8</v>
       </c>
@@ -944,7 +953,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="43" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" ht="42.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>8</v>
       </c>
@@ -961,7 +970,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="43" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" ht="42.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>8</v>
       </c>
@@ -978,7 +987,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="43" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" ht="42.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>8</v>
       </c>
@@ -995,7 +1004,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="43" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" ht="42.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>8</v>
       </c>
@@ -1012,7 +1021,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="43" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" ht="42.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>8</v>
       </c>
@@ -1029,7 +1038,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="43" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" ht="42.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>28</v>
       </c>
@@ -1040,13 +1049,13 @@
         <v>30</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="43" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5" ht="42.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>28</v>
       </c>
@@ -1057,13 +1066,13 @@
         <v>32</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="43" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5" ht="42.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>28</v>
       </c>
@@ -1074,13 +1083,13 @@
         <v>34</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="17" spans="1:5" ht="43" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5" ht="42.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>28</v>
       </c>
@@ -1091,13 +1100,13 @@
         <v>36</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="18" spans="1:5" ht="43" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5" ht="42.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>28</v>
       </c>
@@ -1108,13 +1117,13 @@
         <v>38</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="19" spans="1:5" ht="43" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5" ht="42.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>28</v>
       </c>
@@ -1125,13 +1134,13 @@
         <v>40</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="20" spans="1:5" ht="43" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5" ht="42.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>28</v>
       </c>
@@ -1142,13 +1151,13 @@
         <v>42</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="21" spans="1:5" ht="43" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5" ht="42.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>28</v>
       </c>
@@ -1159,13 +1168,13 @@
         <v>44</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="22" spans="1:5" ht="43" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:5" ht="42.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>46</v>
       </c>
@@ -1182,7 +1191,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="23" spans="1:5" ht="43" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:5" ht="42.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>46</v>
       </c>
@@ -1199,7 +1208,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="24" spans="1:5" ht="43" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:5" ht="42.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>46</v>
       </c>
@@ -1216,7 +1225,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="25" spans="1:5" ht="43" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:5" ht="42.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>46</v>
       </c>
@@ -1233,7 +1242,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="26" spans="1:5" ht="43" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:5" ht="42.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>46</v>
       </c>
@@ -1250,7 +1259,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="27" spans="1:5" ht="43" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:5" ht="42.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>46</v>
       </c>
@@ -1267,7 +1276,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="28" spans="1:5" ht="43" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:5" ht="42.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>46</v>
       </c>
@@ -1284,7 +1293,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="29" spans="1:5" ht="43" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:5" ht="42.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>46</v>
       </c>
@@ -1301,21 +1310,21 @@
         <v>63</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="3"/>
       <c r="B30" s="3"/>
       <c r="C30" s="3"/>
       <c r="D30" s="3"/>
       <c r="E30" s="3"/>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="3"/>
       <c r="B31" s="3"/>
       <c r="C31" s="3"/>
       <c r="D31" s="3"/>
       <c r="E31" s="3"/>
     </row>
-    <row r="32" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="12" t="s">
         <v>64</v>
       </c>
@@ -1324,7 +1333,7 @@
       <c r="D32" s="10"/>
       <c r="E32" s="10"/>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="6" t="s">
         <v>3</v>
       </c>
@@ -1341,7 +1350,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="7" t="s">
         <v>8</v>
       </c>
@@ -1362,7 +1371,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="7" t="s">
         <v>28</v>
       </c>
@@ -1372,7 +1381,7 @@
       </c>
       <c r="C35" s="5">
         <f>COUNTIFS($A$6:$A$29,A35,$D$6:$D$29,"☑ Complete")</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="D35" s="5">
         <f>COUNTIFS($A$6:$A$29,A35,$D$6:$D$29,"◐ In progress")</f>
@@ -1383,7 +1392,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="7" t="s">
         <v>46</v>
       </c>
@@ -1445,7 +1454,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:D13"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="52" customWidth="1"/>
     <col min="2" max="2" width="25" customWidth="1"/>
@@ -1453,7 +1462,7 @@
     <col min="4" max="4" width="38" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="32.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="14" t="s">
         <v>69</v>
       </c>
@@ -1461,7 +1470,7 @@
       <c r="C1" s="10"/>
       <c r="D1" s="10"/>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="15" t="s">
         <v>70</v>
       </c>
@@ -1469,13 +1478,13 @@
       <c r="C2" s="10"/>
       <c r="D2" s="10"/>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="3"/>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
         <v>71</v>
       </c>
@@ -1489,7 +1498,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="38.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" ht="38.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>74</v>
       </c>
@@ -1503,7 +1512,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="38.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" ht="38.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>77</v>
       </c>
@@ -1517,7 +1526,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="38.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" ht="38.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>80</v>
       </c>
@@ -1531,7 +1540,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="38.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" ht="38.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>83</v>
       </c>
@@ -1545,7 +1554,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="38.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" ht="38.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>85</v>
       </c>
@@ -1557,7 +1566,7 @@
       </c>
       <c r="D9" s="2"/>
     </row>
-    <row r="10" spans="1:4" ht="38.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" ht="38.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>87</v>
       </c>
@@ -1569,7 +1578,7 @@
       </c>
       <c r="D10" s="2"/>
     </row>
-    <row r="11" spans="1:4" ht="38.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" ht="38.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>89</v>
       </c>
@@ -1583,7 +1592,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="38.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" ht="38.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>92</v>
       </c>
@@ -1595,7 +1604,7 @@
       </c>
       <c r="D12" s="2"/>
     </row>
-    <row r="13" spans="1:4" ht="38.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" ht="38.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>94</v>
       </c>

</xml_diff>